<commit_message>
submitted to EA cleanup
</commit_message>
<xml_diff>
--- a/03_output/water_analysis/ModelAnalyses.xlsx
+++ b/03_output/water_analysis/ModelAnalyses.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/margaretswift/Documents/03 Science/00 Research - Active/WWF KAZA Waterholes/Rasters/output/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/margaretswift/Documents/03 Science/00 Research - Active/WWF KAZA Waterholes/kaza-water-case-study/03_output/water_analysis/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70545665-209F-2545-B0D9-E9003E90DC7F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4D13E4C-4679-8243-B862-B518101615AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28660" yWindow="3320" windowWidth="28040" windowHeight="17440" activeTab="3" xr2:uid="{B16B2437-0AA4-994C-9210-1E1525A19DED}"/>
+    <workbookView xWindow="-19820" yWindow="2640" windowWidth="21600" windowHeight="17440" xr2:uid="{B16B2437-0AA4-994C-9210-1E1525A19DED}"/>
   </bookViews>
   <sheets>
-    <sheet name="Tukey HSD Hydrosheds" sheetId="1" r:id="rId1"/>
-    <sheet name="Tukey HSD SIZ" sheetId="3" r:id="rId2"/>
-    <sheet name="GLMM Results" sheetId="6" r:id="rId3"/>
-    <sheet name="GLMM Results 2" sheetId="5" r:id="rId4"/>
+    <sheet name="KW" sheetId="7" r:id="rId1"/>
+    <sheet name="Tukey HSD Hydrosheds" sheetId="1" r:id="rId2"/>
+    <sheet name="Tukey HSD SIZ" sheetId="3" r:id="rId3"/>
+    <sheet name="GLMM Results" sheetId="6" r:id="rId4"/>
+    <sheet name="GLMM Results 2" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -39,7 +40,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="89" uniqueCount="46">
   <si>
     <t>FEB_MAY-NOV_FEB</t>
   </si>
@@ -183,6 +184,21 @@
   </si>
   <si>
     <t>&lt;&lt; 0.01</t>
+  </si>
+  <si>
+    <t>Nov - Feb</t>
+  </si>
+  <si>
+    <t>Feb - May</t>
+  </si>
+  <si>
+    <t>May - July</t>
+  </si>
+  <si>
+    <t>July - Sept</t>
+  </si>
+  <si>
+    <t>Sept - Nov</t>
   </si>
 </sst>
 </file>
@@ -258,7 +274,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="11" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -280,6 +296,12 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -614,6 +636,83 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9B19344A-A693-D442-9C28-AFF1A1DC2C14}">
+  <dimension ref="A1:E5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="5" width="10.83203125" style="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="B1" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D1" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E1" s="12" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A2" t="s">
+        <v>42</v>
+      </c>
+      <c r="B2" s="13" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A3" t="s">
+        <v>43</v>
+      </c>
+      <c r="B3" s="12">
+        <v>0.25</v>
+      </c>
+      <c r="C3" s="13" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="12">
+        <v>1</v>
+      </c>
+      <c r="C4" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="D4" s="12">
+        <v>1.7999999999999999E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B5" s="12">
+        <v>5.6000000000000001E-2</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="E5" s="12">
+        <v>0.47599999999999998</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{595288FF-18B8-9B4D-A497-14C9EA5BD57C}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -814,7 +913,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B3B7C534-28EF-7F43-843B-065C4D79DFE9}">
   <dimension ref="A1:E11"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1011,7 +1110,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8A5B6C9E-788B-B840-9C68-DC844973B3A9}">
   <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
@@ -1387,7 +1486,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7D34EEBE-66C2-8445-B6DB-D2BD396C8464}">
   <dimension ref="A1:F21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>